<commit_message>
Rework Doft Diwali pop-up brief response: ProMarcom pitch deck + costing workbook
- Add ProMarcom-branded pitch deck (17 slides) replacing the Word plan
- Rebrand operations & costing workbook to ProMarcom
- Remove retired Word execution plan and its build script

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SPjFYHW1nTDVr5tUuToRXR
</commit_message>
<xml_diff>
--- a/doft_diwali_popup/Doft_Diwali_PopUp_Operations_Workbook.xlsx
+++ b/doft_diwali_popup/Doft_Diwali_PopUp_Operations_Workbook.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="1. README &amp; Assumptions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2. Project Timeline" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="3. Staffing Plan" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="4. Manpower Cost" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="5. Budget Summary" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="6. Recruitment Tracker" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="7. Attendance Tracker" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="8. Daily Sales Report" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="9. Inventory &amp; Replenish" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="10. Footfall &amp; Conversion" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="11. Customer Feedback" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="12. Compliance Checklist" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="13. Risk Register" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. README &amp; Assumptions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Project Timeline" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Staffing Plan" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Manpower Cost" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Budget Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. Recruitment Tracker" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. Attendance Tracker" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. Daily Sales Report" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. Inventory &amp; Replenish" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. Footfall &amp; Conversion" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11. Customer Feedback" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12. Compliance Checklist" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13. Risk Register" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -881,7 +881,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Contractor Operations &amp; Costing Workbook  |  Seasons 2026 / 2027 / 2028</t>
+          <t>ProMarcom Inc.  |  Operations &amp; Costing Workbook  |  Seasons 2026 / 2027 / 2028</t>
         </is>
       </c>
     </row>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="F5" s="28" t="inlineStr">
         <is>
-          <t>Contractor payroll</t>
+          <t>ProMarcom payroll</t>
         </is>
       </c>
     </row>
@@ -3307,7 +3307,7 @@
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Contractor payroll</t>
+          <t>ProMarcom payroll</t>
         </is>
       </c>
     </row>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="F7" s="28" t="inlineStr">
         <is>
-          <t>Contractor payroll</t>
+          <t>ProMarcom payroll</t>
         </is>
       </c>
     </row>
@@ -3367,7 +3367,7 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Contractor payroll</t>
+          <t>ProMarcom payroll</t>
         </is>
       </c>
     </row>
@@ -3397,7 +3397,7 @@
       </c>
       <c r="F9" s="28" t="inlineStr">
         <is>
-          <t>Contractor payroll</t>
+          <t>ProMarcom payroll</t>
         </is>
       </c>
     </row>

</xml_diff>